<commit_message>
Use the real Sheet 3 rate card and skip the template's example row
Three carriers per route (A economy, B standard 750 kg, C express) copied
from Case2_Shipment_Booking_Test_Data_Format.xlsx. Uploads ignore the grey
example row only when it is left exactly as shipped. Sample workbook
updated so each planted mistake still trips against the real card.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/sample-shipments.xlsx
+++ b/public/sample-shipments.xlsx
@@ -497,7 +497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BK-001</t>
+          <t>BK-006</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>650</v>
+        <v>800</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BK-001</t>
+          <t>BK-006</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>